<commit_message>
Make per-ID selection robust to repeated IDs and price ties
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFaw3CrmucU3qXrStYrfnC
</commit_message>
<xml_diff>
--- a/Выбор_по_договору_ID.xlsx
+++ b/Выбор_по_договору_ID.xlsx
@@ -138,12 +138,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -412,432 +416,432 @@
   <dimension ref="M1:T17"/>
   <sheetFormatPr defaultColWidth="8.55859375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="9.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="19.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="23.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="36.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="35.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="11.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="9.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="19.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="12.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="23.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="36.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="35.89"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="M1" s="0" t="s">
+      <c r="M1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="N1" s="0" t="s">
+      <c r="N1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="O1" s="0" t="s">
+      <c r="O1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="0" t="s">
+      <c r="P1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="0" t="s">
+      <c r="Q1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="R1" s="0" t="s">
+      <c r="R1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="S1" s="0" t="s">
+      <c r="S1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="M2" s="0" t="n">
+      <c r="M2" s="1" t="n">
         <v>99008177</v>
       </c>
-      <c r="N2" s="0" t="n">
+      <c r="N2" s="1" t="n">
         <v>147185</v>
       </c>
-      <c r="O2" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P2" s="0" t="s">
+      <c r="O2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="Q2" s="0" t="n">
+      <c r="Q2" s="1" t="n">
         <v>3772.23</v>
       </c>
-      <c r="R2" s="0" t="n">
+      <c r="R2" s="1" t="n">
         <v>242</v>
       </c>
-      <c r="S2" s="0" t="n">
+      <c r="S2" s="1" t="n">
         <v>158</v>
       </c>
-      <c r="T2" s="0" t="str">
-        <f aca="false">IF(AND(OR(P2="RAM",P2="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M2&lt;&gt;""),ROW($M$2:M2)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M3:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q2))=0),"Выбрать","")</f>
+      <c r="T2" s="1" t="str">
+        <f aca="false">IF(AND(OR(P2="RAM",P2="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M1&lt;&gt;"")*($M$1:M1&lt;&gt;LOOKUP(2,1/($M$2:M2&lt;&gt;""),$M$2:M2))),ROW($M$1:M1))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M3:$M$1001&lt;&gt;"")*(M3:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M2&lt;&gt;""),$M$2:M2)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q2)+($Q$2:$Q$1000=Q2)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="N3" s="0" t="n">
+      <c r="N3" s="1" t="n">
         <v>298654</v>
       </c>
-      <c r="O3" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P3" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q3" s="0" t="n">
+      <c r="O3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q3" s="1" t="n">
         <v>594.94</v>
       </c>
-      <c r="R3" s="0" t="n">
+      <c r="R3" s="1" t="n">
         <v>212</v>
       </c>
-      <c r="S3" s="0" t="n">
+      <c r="S3" s="1" t="n">
         <v>128</v>
       </c>
-      <c r="T3" s="0" t="str">
-        <f aca="false">IF(AND(OR(P3="RAM",P3="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M3&lt;&gt;""),ROW($M$2:M3)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M4:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q3))=0),"Выбрать","")</f>
+      <c r="T3" s="1" t="str">
+        <f aca="false">IF(AND(OR(P3="RAM",P3="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M2&lt;&gt;"")*($M$1:M2&lt;&gt;LOOKUP(2,1/($M$2:M3&lt;&gt;""),$M$2:M3))),ROW($M$1:M2))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M4:$M$1001&lt;&gt;"")*(M4:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M3&lt;&gt;""),$M$2:M3)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q3)+($Q$2:$Q$1000=Q3)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="N4" s="0" t="n">
+      <c r="N4" s="1" t="n">
         <v>298733</v>
       </c>
-      <c r="O4" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P4" s="0" t="s">
+      <c r="O4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Q4" s="0" t="n">
+      <c r="Q4" s="1" t="n">
         <v>765.36</v>
       </c>
-      <c r="R4" s="0" t="n">
+      <c r="R4" s="1" t="n">
         <v>143</v>
       </c>
-      <c r="S4" s="0" t="n">
+      <c r="S4" s="1" t="n">
         <v>59</v>
       </c>
-      <c r="T4" s="0" t="str">
-        <f aca="false">IF(AND(OR(P4="RAM",P4="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M4&lt;&gt;""),ROW($M$2:M4)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M5:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q4))=0),"Выбрать","")</f>
+      <c r="T4" s="1" t="str">
+        <f aca="false">IF(AND(OR(P4="RAM",P4="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M3&lt;&gt;"")*($M$1:M3&lt;&gt;LOOKUP(2,1/($M$2:M4&lt;&gt;""),$M$2:M4))),ROW($M$1:M3))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M5:$M$1001&lt;&gt;"")*(M5:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M4&lt;&gt;""),$M$2:M4)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q4)+($Q$2:$Q$1000=Q4)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
         <v>Выбрать</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="N5" s="0" t="n">
+      <c r="N5" s="1" t="n">
         <v>508788</v>
       </c>
-      <c r="O5" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P5" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q5" s="0" t="n">
+      <c r="O5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q5" s="1" t="n">
         <v>368.56</v>
       </c>
-      <c r="R5" s="0" t="n">
+      <c r="R5" s="1" t="n">
         <v>202</v>
       </c>
-      <c r="S5" s="0" t="n">
+      <c r="S5" s="1" t="n">
         <v>118</v>
       </c>
-      <c r="T5" s="0" t="str">
-        <f aca="false">IF(AND(OR(P5="RAM",P5="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M5&lt;&gt;""),ROW($M$2:M5)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M6:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q5))=0),"Выбрать","")</f>
+      <c r="T5" s="1" t="str">
+        <f aca="false">IF(AND(OR(P5="RAM",P5="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M4&lt;&gt;"")*($M$1:M4&lt;&gt;LOOKUP(2,1/($M$2:M5&lt;&gt;""),$M$2:M5))),ROW($M$1:M4))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M6:$M$1001&lt;&gt;"")*(M6:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M5&lt;&gt;""),$M$2:M5)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q5)+($Q$2:$Q$1000=Q5)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="N6" s="0" t="n">
+      <c r="N6" s="1" t="n">
         <v>509811</v>
       </c>
-      <c r="O6" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P6" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q6" s="0" t="n">
+      <c r="O6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q6" s="1" t="n">
         <v>873.5</v>
       </c>
-      <c r="R6" s="0" t="n">
+      <c r="R6" s="1" t="n">
         <v>165</v>
       </c>
-      <c r="S6" s="0" t="n">
+      <c r="S6" s="1" t="n">
         <v>81</v>
       </c>
-      <c r="T6" s="0" t="str">
-        <f aca="false">IF(AND(OR(P6="RAM",P6="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M6&lt;&gt;""),ROW($M$2:M6)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M7:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q6))=0),"Выбрать","")</f>
+      <c r="T6" s="1" t="str">
+        <f aca="false">IF(AND(OR(P6="RAM",P6="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M5&lt;&gt;"")*($M$1:M5&lt;&gt;LOOKUP(2,1/($M$2:M6&lt;&gt;""),$M$2:M6))),ROW($M$1:M5))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M7:$M$1001&lt;&gt;"")*(M7:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M6&lt;&gt;""),$M$2:M6)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q6)+($Q$2:$Q$1000=Q6)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="N7" s="0" t="n">
+      <c r="N7" s="1" t="n">
         <v>519150</v>
       </c>
-      <c r="O7" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P7" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q7" s="0" t="n">
+      <c r="O7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q7" s="1" t="n">
         <v>1229.03</v>
       </c>
-      <c r="R7" s="0" t="n">
+      <c r="R7" s="1" t="n">
         <v>202</v>
       </c>
-      <c r="S7" s="0" t="n">
+      <c r="S7" s="1" t="n">
         <v>118</v>
       </c>
-      <c r="T7" s="0" t="str">
-        <f aca="false">IF(AND(OR(P7="RAM",P7="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M7&lt;&gt;""),ROW($M$2:M7)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M8:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q7))=0),"Выбрать","")</f>
+      <c r="T7" s="1" t="str">
+        <f aca="false">IF(AND(OR(P7="RAM",P7="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M6&lt;&gt;"")*($M$1:M6&lt;&gt;LOOKUP(2,1/($M$2:M7&lt;&gt;""),$M$2:M7))),ROW($M$1:M6))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M8:$M$1001&lt;&gt;"")*(M8:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M7&lt;&gt;""),$M$2:M7)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q7)+($Q$2:$Q$1000=Q7)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="N8" s="0" t="n">
+      <c r="N8" s="1" t="n">
         <v>526401</v>
       </c>
-      <c r="O8" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P8" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q8" s="0" t="n">
+      <c r="O8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q8" s="1" t="n">
         <v>752.39</v>
       </c>
-      <c r="R8" s="0" t="n">
+      <c r="R8" s="1" t="n">
         <v>212</v>
       </c>
-      <c r="S8" s="0" t="n">
+      <c r="S8" s="1" t="n">
         <v>128</v>
       </c>
-      <c r="T8" s="0" t="str">
-        <f aca="false">IF(AND(OR(P8="RAM",P8="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M8&lt;&gt;""),ROW($M$2:M8)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M9:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q8))=0),"Выбрать","")</f>
+      <c r="T8" s="1" t="str">
+        <f aca="false">IF(AND(OR(P8="RAM",P8="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M7&lt;&gt;"")*($M$1:M7&lt;&gt;LOOKUP(2,1/($M$2:M8&lt;&gt;""),$M$2:M8))),ROW($M$1:M7))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M9:$M$1001&lt;&gt;"")*(M9:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M8&lt;&gt;""),$M$2:M8)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q8)+($Q$2:$Q$1000=Q8)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="N9" s="0" t="n">
+      <c r="N9" s="1" t="n">
         <v>1520422</v>
       </c>
-      <c r="O9" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P9" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q9" s="0" t="n">
+      <c r="O9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q9" s="1" t="n">
         <v>2735.52</v>
       </c>
-      <c r="R9" s="0" t="e">
+      <c r="R9" s="1" t="e">
         <f aca="false">#N/A</f>
         <v>#N/A</v>
       </c>
-      <c r="S9" s="0" t="e">
+      <c r="S9" s="1" t="e">
         <f aca="false">#N/A</f>
         <v>#N/A</v>
       </c>
-      <c r="T9" s="0" t="str">
-        <f aca="false">IF(AND(OR(P9="RAM",P9="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M9&lt;&gt;""),ROW($M$2:M9)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M10:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q9))=0),"Выбрать","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M10" s="0" t="n">
+      <c r="T9" s="1" t="str">
+        <f aca="false">IF(AND(OR(P9="RAM",P9="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M8&lt;&gt;"")*($M$1:M8&lt;&gt;LOOKUP(2,1/($M$2:M9&lt;&gt;""),$M$2:M9))),ROW($M$1:M8))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M10:$M$1001&lt;&gt;"")*(M10:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M9&lt;&gt;""),$M$2:M9)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q9)+($Q$2:$Q$1000=Q9)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M10" s="1" t="n">
         <v>99008188</v>
       </c>
-      <c r="N10" s="0" t="n">
+      <c r="N10" s="1" t="n">
         <v>254877</v>
       </c>
-      <c r="O10" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P10" s="0" t="s">
+      <c r="O10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="Q10" s="0" t="n">
+      <c r="Q10" s="1" t="n">
         <v>3772.23</v>
       </c>
-      <c r="R10" s="0" t="n">
+      <c r="R10" s="1" t="n">
         <v>242</v>
       </c>
-      <c r="S10" s="0" t="n">
+      <c r="S10" s="1" t="n">
         <v>158</v>
       </c>
-      <c r="T10" s="0" t="str">
-        <f aca="false">IF(AND(OR(P10="RAM",P10="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M10&lt;&gt;""),ROW($M$2:M10)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M11:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q10))=0),"Выбрать","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N11" s="0" t="n">
+      <c r="T10" s="1" t="str">
+        <f aca="false">IF(AND(OR(P10="RAM",P10="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M9&lt;&gt;"")*($M$1:M9&lt;&gt;LOOKUP(2,1/($M$2:M10&lt;&gt;""),$M$2:M10))),ROW($M$1:M9))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M11:$M$1001&lt;&gt;"")*(M11:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M10&lt;&gt;""),$M$2:M10)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q10)+($Q$2:$Q$1000=Q10)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N11" s="1" t="n">
         <v>1487522</v>
       </c>
-      <c r="O11" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P11" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q11" s="0" t="n">
+      <c r="O11" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q11" s="1" t="n">
         <v>594.94</v>
       </c>
-      <c r="R11" s="0" t="n">
+      <c r="R11" s="1" t="n">
         <v>212</v>
       </c>
-      <c r="S11" s="0" t="n">
+      <c r="S11" s="1" t="n">
         <v>128</v>
       </c>
-      <c r="T11" s="0" t="str">
-        <f aca="false">IF(AND(OR(P11="RAM",P11="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M11&lt;&gt;""),ROW($M$2:M11)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M12:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q11))=0),"Выбрать","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N12" s="0" t="n">
+      <c r="T11" s="1" t="str">
+        <f aca="false">IF(AND(OR(P11="RAM",P11="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M10&lt;&gt;"")*($M$1:M10&lt;&gt;LOOKUP(2,1/($M$2:M11&lt;&gt;""),$M$2:M11))),ROW($M$1:M10))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M12:$M$1001&lt;&gt;"")*(M12:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M11&lt;&gt;""),$M$2:M11)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q11)+($Q$2:$Q$1000=Q11)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N12" s="1" t="n">
         <v>145211</v>
       </c>
-      <c r="O12" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P12" s="0" t="s">
+      <c r="O12" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Q12" s="0" t="n">
+      <c r="Q12" s="1" t="n">
         <v>1565.36</v>
       </c>
-      <c r="R12" s="0" t="n">
+      <c r="R12" s="1" t="n">
         <v>143</v>
       </c>
-      <c r="S12" s="0" t="n">
+      <c r="S12" s="1" t="n">
         <v>59</v>
       </c>
-      <c r="T12" s="0" t="str">
-        <f aca="false">IF(AND(OR(P12="RAM",P12="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M12&lt;&gt;""),ROW($M$2:M12)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M13:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q12))=0),"Выбрать","")</f>
-        <v>Выбрать</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N13" s="0" t="n">
+      <c r="T12" s="1" t="str">
+        <f aca="false">IF(AND(OR(P12="RAM",P12="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M11&lt;&gt;"")*($M$1:M11&lt;&gt;LOOKUP(2,1/($M$2:M12&lt;&gt;""),$M$2:M12))),ROW($M$1:M11))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M13:$M$1001&lt;&gt;"")*(M13:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M12&lt;&gt;""),$M$2:M12)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q12)+($Q$2:$Q$1000=Q12)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N13" s="1" t="n">
         <v>1177852</v>
       </c>
-      <c r="O13" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P13" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q13" s="0" t="n">
+      <c r="O13" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q13" s="1" t="n">
         <v>368.56</v>
       </c>
-      <c r="R13" s="0" t="n">
+      <c r="R13" s="1" t="n">
         <v>202</v>
       </c>
-      <c r="S13" s="0" t="n">
+      <c r="S13" s="1" t="n">
         <v>118</v>
       </c>
-      <c r="T13" s="0" t="str">
-        <f aca="false">IF(AND(OR(P13="RAM",P13="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M13&lt;&gt;""),ROW($M$2:M13)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M14:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q13))=0),"Выбрать","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N14" s="0" t="n">
+      <c r="T13" s="1" t="str">
+        <f aca="false">IF(AND(OR(P13="RAM",P13="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M12&lt;&gt;"")*($M$1:M12&lt;&gt;LOOKUP(2,1/($M$2:M13&lt;&gt;""),$M$2:M13))),ROW($M$1:M12))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M14:$M$1001&lt;&gt;"")*(M14:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M13&lt;&gt;""),$M$2:M13)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q13)+($Q$2:$Q$1000=Q13)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N14" s="1" t="n">
         <v>445221</v>
       </c>
-      <c r="O14" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P14" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q14" s="0" t="n">
+      <c r="O14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q14" s="1" t="n">
         <v>873.5</v>
       </c>
-      <c r="R14" s="0" t="n">
+      <c r="R14" s="1" t="n">
         <v>165</v>
       </c>
-      <c r="S14" s="0" t="n">
+      <c r="S14" s="1" t="n">
         <v>81</v>
       </c>
-      <c r="T14" s="0" t="str">
-        <f aca="false">IF(AND(OR(P14="RAM",P14="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M14&lt;&gt;""),ROW($M$2:M14)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M15:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q14))=0),"Выбрать","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N15" s="0" t="n">
+      <c r="T14" s="1" t="str">
+        <f aca="false">IF(AND(OR(P14="RAM",P14="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M13&lt;&gt;"")*($M$1:M13&lt;&gt;LOOKUP(2,1/($M$2:M14&lt;&gt;""),$M$2:M14))),ROW($M$1:M13))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M15:$M$1001&lt;&gt;"")*(M15:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M14&lt;&gt;""),$M$2:M14)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q14)+($Q$2:$Q$1000=Q14)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N15" s="1" t="n">
         <v>441155</v>
       </c>
-      <c r="O15" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P15" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q15" s="0" t="n">
+      <c r="O15" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q15" s="1" t="n">
         <v>1229.03</v>
       </c>
-      <c r="R15" s="0" t="n">
+      <c r="R15" s="1" t="n">
         <v>202</v>
       </c>
-      <c r="S15" s="0" t="n">
+      <c r="S15" s="1" t="n">
         <v>118</v>
       </c>
-      <c r="T15" s="0" t="str">
-        <f aca="false">IF(AND(OR(P15="RAM",P15="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M15&lt;&gt;""),ROW($M$2:M15)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M16:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q15))=0),"Выбрать","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N16" s="0" t="n">
+      <c r="T15" s="1" t="str">
+        <f aca="false">IF(AND(OR(P15="RAM",P15="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M14&lt;&gt;"")*($M$1:M14&lt;&gt;LOOKUP(2,1/($M$2:M15&lt;&gt;""),$M$2:M15))),ROW($M$1:M14))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M16:$M$1001&lt;&gt;"")*(M16:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M15&lt;&gt;""),$M$2:M15)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q15)+($Q$2:$Q$1000=Q15)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N16" s="1" t="n">
         <v>155221</v>
       </c>
-      <c r="O16" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P16" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q16" s="0" t="n">
+      <c r="O16" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q16" s="1" t="n">
         <v>752.39</v>
       </c>
-      <c r="R16" s="0" t="n">
+      <c r="R16" s="1" t="n">
         <v>212</v>
       </c>
-      <c r="S16" s="0" t="n">
+      <c r="S16" s="1" t="n">
         <v>128</v>
       </c>
-      <c r="T16" s="0" t="str">
-        <f aca="false">IF(AND(OR(P16="RAM",P16="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M16&lt;&gt;""),ROW($M$2:M16)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M17:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q16))=0),"Выбрать","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N17" s="0" t="n">
+      <c r="T16" s="1" t="str">
+        <f aca="false">IF(AND(OR(P16="RAM",P16="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M15&lt;&gt;"")*($M$1:M15&lt;&gt;LOOKUP(2,1/($M$2:M16&lt;&gt;""),$M$2:M16))),ROW($M$1:M15))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M17:$M$1001&lt;&gt;"")*(M17:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M16&lt;&gt;""),$M$2:M16)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q16)+($Q$2:$Q$1000=Q16)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N17" s="1" t="n">
         <v>5444445</v>
       </c>
-      <c r="O17" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="P17" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q17" s="0" t="n">
+      <c r="O17" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q17" s="1" t="n">
         <v>2735.52</v>
       </c>
-      <c r="R17" s="0" t="e">
+      <c r="R17" s="1" t="e">
         <f aca="false">#N/A</f>
         <v>#N/A</v>
       </c>
-      <c r="S17" s="0" t="e">
+      <c r="S17" s="1" t="e">
         <f aca="false">#N/A</f>
         <v>#N/A</v>
       </c>
-      <c r="T17" s="0" t="str">
-        <f aca="false">IF(AND(OR(P17="RAM",P17="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=LOOKUP(2,1/($M$2:M17&lt;&gt;""),ROW($M$2:M17)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(TRUE(),INDEX(M18:$M$1001&lt;&gt;"",0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*($Q$2:$Q$1000&lt;Q17))=0),"Выбрать","")</f>
+      <c r="T17" s="1" t="str">
+        <f aca="false">IF(AND(OR(P17="RAM",P17="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=IFERROR(LOOKUP(2,1/(($M$1:M16&lt;&gt;"")*($M$1:M16&lt;&gt;LOOKUP(2,1/($M$2:M17&lt;&gt;""),$M$2:M17))),ROW($M$1:M16))+1,2))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M18:$M$1001&lt;&gt;"")*(M18:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M17&lt;&gt;""),$M$2:M17)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q17)+($Q$2:$Q$1000=Q17)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Switch to ID-per-row layout with short COUNTIFS selection formula
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFaw3CrmucU3qXrStYrfnC
</commit_message>
<xml_diff>
--- a/Выбор_по_договору_ID.xlsx
+++ b/Выбор_по_договору_ID.xlsx
@@ -474,11 +474,14 @@
         <v>158</v>
       </c>
       <c r="T2" s="1" t="str">
-        <f aca="false">IF(AND(OR(P2="RAM",P2="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M1&lt;&gt;"")*($M$1:M1&lt;&gt;LOOKUP(2,1/($M$2:M2&lt;&gt;""),$M$2:M2))),ROW($M$1:M1)),1)+MATCH(LOOKUP(2,1/($M$2:M2&lt;&gt;""),$M$2:M2),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M1&lt;&gt;"")*($M$1:M1&lt;&gt;LOOKUP(2,1/($M$2:M2&lt;&gt;""),$M$2:M2))),ROW($M$1:M1)),1)+1):M2,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M3:$M$1001&lt;&gt;"")*(M3:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M2&lt;&gt;""),$M$2:M2)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q2)+($Q$2:$Q$1000=Q2)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P2="RAM",P2="KON"),COUNTIFS($M$2:$M$1000,M2,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q2)+COUNTIFS($M$1:M1,M2,$P$1:P1,"RAM",$Q$1:Q1,Q2)+COUNTIFS($M$2:$M$1000,M2,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q2)+COUNTIFS($M$1:M1,M2,$P$1:P1,"KON",$Q$1:Q1,Q2)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M3" s="1" t="n">
+        <v>99008177</v>
+      </c>
       <c r="N3" s="1" t="n">
         <v>298654</v>
       </c>
@@ -498,11 +501,14 @@
         <v>128</v>
       </c>
       <c r="T3" s="1" t="str">
-        <f aca="false">IF(AND(OR(P3="RAM",P3="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M2&lt;&gt;"")*($M$1:M2&lt;&gt;LOOKUP(2,1/($M$2:M3&lt;&gt;""),$M$2:M3))),ROW($M$1:M2)),1)+MATCH(LOOKUP(2,1/($M$2:M3&lt;&gt;""),$M$2:M3),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M2&lt;&gt;"")*($M$1:M2&lt;&gt;LOOKUP(2,1/($M$2:M3&lt;&gt;""),$M$2:M3))),ROW($M$1:M2)),1)+1):M3,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M4:$M$1001&lt;&gt;"")*(M4:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M3&lt;&gt;""),$M$2:M3)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q3)+($Q$2:$Q$1000=Q3)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P3="RAM",P3="KON"),COUNTIFS($M$2:$M$1000,M3,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q3)+COUNTIFS($M$1:M2,M3,$P$1:P2,"RAM",$Q$1:Q2,Q3)+COUNTIFS($M$2:$M$1000,M3,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q3)+COUNTIFS($M$1:M2,M3,$P$1:P2,"KON",$Q$1:Q2,Q3)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M4" s="1" t="n">
+        <v>99008177</v>
+      </c>
       <c r="N4" s="1" t="n">
         <v>298733</v>
       </c>
@@ -522,11 +528,14 @@
         <v>59</v>
       </c>
       <c r="T4" s="1" t="str">
-        <f aca="false">IF(AND(OR(P4="RAM",P4="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M3&lt;&gt;"")*($M$1:M3&lt;&gt;LOOKUP(2,1/($M$2:M4&lt;&gt;""),$M$2:M4))),ROW($M$1:M3)),1)+MATCH(LOOKUP(2,1/($M$2:M4&lt;&gt;""),$M$2:M4),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M3&lt;&gt;"")*($M$1:M3&lt;&gt;LOOKUP(2,1/($M$2:M4&lt;&gt;""),$M$2:M4))),ROW($M$1:M3)),1)+1):M4,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M5:$M$1001&lt;&gt;"")*(M5:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M4&lt;&gt;""),$M$2:M4)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q4)+($Q$2:$Q$1000=Q4)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P4="RAM",P4="KON"),COUNTIFS($M$2:$M$1000,M4,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q4)+COUNTIFS($M$1:M3,M4,$P$1:P3,"RAM",$Q$1:Q3,Q4)+COUNTIFS($M$2:$M$1000,M4,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q4)+COUNTIFS($M$1:M3,M4,$P$1:P3,"KON",$Q$1:Q3,Q4)=0),"Выбрать","")</f>
         <v>Выбрать</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M5" s="1" t="n">
+        <v>99008177</v>
+      </c>
       <c r="N5" s="1" t="n">
         <v>508788</v>
       </c>
@@ -546,11 +555,14 @@
         <v>118</v>
       </c>
       <c r="T5" s="1" t="str">
-        <f aca="false">IF(AND(OR(P5="RAM",P5="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M4&lt;&gt;"")*($M$1:M4&lt;&gt;LOOKUP(2,1/($M$2:M5&lt;&gt;""),$M$2:M5))),ROW($M$1:M4)),1)+MATCH(LOOKUP(2,1/($M$2:M5&lt;&gt;""),$M$2:M5),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M4&lt;&gt;"")*($M$1:M4&lt;&gt;LOOKUP(2,1/($M$2:M5&lt;&gt;""),$M$2:M5))),ROW($M$1:M4)),1)+1):M5,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M6:$M$1001&lt;&gt;"")*(M6:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M5&lt;&gt;""),$M$2:M5)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q5)+($Q$2:$Q$1000=Q5)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P5="RAM",P5="KON"),COUNTIFS($M$2:$M$1000,M5,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q5)+COUNTIFS($M$1:M4,M5,$P$1:P4,"RAM",$Q$1:Q4,Q5)+COUNTIFS($M$2:$M$1000,M5,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q5)+COUNTIFS($M$1:M4,M5,$P$1:P4,"KON",$Q$1:Q4,Q5)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M6" s="1" t="n">
+        <v>99008177</v>
+      </c>
       <c r="N6" s="1" t="n">
         <v>509811</v>
       </c>
@@ -570,11 +582,14 @@
         <v>81</v>
       </c>
       <c r="T6" s="1" t="str">
-        <f aca="false">IF(AND(OR(P6="RAM",P6="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M5&lt;&gt;"")*($M$1:M5&lt;&gt;LOOKUP(2,1/($M$2:M6&lt;&gt;""),$M$2:M6))),ROW($M$1:M5)),1)+MATCH(LOOKUP(2,1/($M$2:M6&lt;&gt;""),$M$2:M6),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M5&lt;&gt;"")*($M$1:M5&lt;&gt;LOOKUP(2,1/($M$2:M6&lt;&gt;""),$M$2:M6))),ROW($M$1:M5)),1)+1):M6,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M7:$M$1001&lt;&gt;"")*(M7:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M6&lt;&gt;""),$M$2:M6)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q6)+($Q$2:$Q$1000=Q6)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P6="RAM",P6="KON"),COUNTIFS($M$2:$M$1000,M6,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q6)+COUNTIFS($M$1:M5,M6,$P$1:P5,"RAM",$Q$1:Q5,Q6)+COUNTIFS($M$2:$M$1000,M6,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q6)+COUNTIFS($M$1:M5,M6,$P$1:P5,"KON",$Q$1:Q5,Q6)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M7" s="1" t="n">
+        <v>99008177</v>
+      </c>
       <c r="N7" s="1" t="n">
         <v>519150</v>
       </c>
@@ -594,11 +609,14 @@
         <v>118</v>
       </c>
       <c r="T7" s="1" t="str">
-        <f aca="false">IF(AND(OR(P7="RAM",P7="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M6&lt;&gt;"")*($M$1:M6&lt;&gt;LOOKUP(2,1/($M$2:M7&lt;&gt;""),$M$2:M7))),ROW($M$1:M6)),1)+MATCH(LOOKUP(2,1/($M$2:M7&lt;&gt;""),$M$2:M7),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M6&lt;&gt;"")*($M$1:M6&lt;&gt;LOOKUP(2,1/($M$2:M7&lt;&gt;""),$M$2:M7))),ROW($M$1:M6)),1)+1):M7,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M8:$M$1001&lt;&gt;"")*(M8:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M7&lt;&gt;""),$M$2:M7)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q7)+($Q$2:$Q$1000=Q7)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P7="RAM",P7="KON"),COUNTIFS($M$2:$M$1000,M7,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q7)+COUNTIFS($M$1:M6,M7,$P$1:P6,"RAM",$Q$1:Q6,Q7)+COUNTIFS($M$2:$M$1000,M7,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q7)+COUNTIFS($M$1:M6,M7,$P$1:P6,"KON",$Q$1:Q6,Q7)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M8" s="1" t="n">
+        <v>99008177</v>
+      </c>
       <c r="N8" s="1" t="n">
         <v>526401</v>
       </c>
@@ -618,11 +636,14 @@
         <v>128</v>
       </c>
       <c r="T8" s="1" t="str">
-        <f aca="false">IF(AND(OR(P8="RAM",P8="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M7&lt;&gt;"")*($M$1:M7&lt;&gt;LOOKUP(2,1/($M$2:M8&lt;&gt;""),$M$2:M8))),ROW($M$1:M7)),1)+MATCH(LOOKUP(2,1/($M$2:M8&lt;&gt;""),$M$2:M8),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M7&lt;&gt;"")*($M$1:M7&lt;&gt;LOOKUP(2,1/($M$2:M8&lt;&gt;""),$M$2:M8))),ROW($M$1:M7)),1)+1):M8,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M9:$M$1001&lt;&gt;"")*(M9:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M8&lt;&gt;""),$M$2:M8)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q8)+($Q$2:$Q$1000=Q8)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P8="RAM",P8="KON"),COUNTIFS($M$2:$M$1000,M8,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q8)+COUNTIFS($M$1:M7,M8,$P$1:P7,"RAM",$Q$1:Q7,Q8)+COUNTIFS($M$2:$M$1000,M8,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q8)+COUNTIFS($M$1:M7,M8,$P$1:P7,"KON",$Q$1:Q7,Q8)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M9" s="1" t="n">
+        <v>99008177</v>
+      </c>
       <c r="N9" s="1" t="n">
         <v>1520422</v>
       </c>
@@ -644,7 +665,7 @@
         <v>#N/A</v>
       </c>
       <c r="T9" s="1" t="str">
-        <f aca="false">IF(AND(OR(P9="RAM",P9="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M8&lt;&gt;"")*($M$1:M8&lt;&gt;LOOKUP(2,1/($M$2:M9&lt;&gt;""),$M$2:M9))),ROW($M$1:M8)),1)+MATCH(LOOKUP(2,1/($M$2:M9&lt;&gt;""),$M$2:M9),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M8&lt;&gt;"")*($M$1:M8&lt;&gt;LOOKUP(2,1/($M$2:M9&lt;&gt;""),$M$2:M9))),ROW($M$1:M8)),1)+1):M9,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M10:$M$1001&lt;&gt;"")*(M10:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M9&lt;&gt;""),$M$2:M9)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q9)+($Q$2:$Q$1000=Q9)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P9="RAM",P9="KON"),COUNTIFS($M$2:$M$1000,M9,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q9)+COUNTIFS($M$1:M8,M9,$P$1:P8,"RAM",$Q$1:Q8,Q9)+COUNTIFS($M$2:$M$1000,M9,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q9)+COUNTIFS($M$1:M8,M9,$P$1:P8,"KON",$Q$1:Q8,Q9)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
@@ -671,11 +692,14 @@
         <v>158</v>
       </c>
       <c r="T10" s="1" t="str">
-        <f aca="false">IF(AND(OR(P10="RAM",P10="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M9&lt;&gt;"")*($M$1:M9&lt;&gt;LOOKUP(2,1/($M$2:M10&lt;&gt;""),$M$2:M10))),ROW($M$1:M9)),1)+MATCH(LOOKUP(2,1/($M$2:M10&lt;&gt;""),$M$2:M10),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M9&lt;&gt;"")*($M$1:M9&lt;&gt;LOOKUP(2,1/($M$2:M10&lt;&gt;""),$M$2:M10))),ROW($M$1:M9)),1)+1):M10,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M11:$M$1001&lt;&gt;"")*(M11:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M10&lt;&gt;""),$M$2:M10)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q10)+($Q$2:$Q$1000=Q10)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P10="RAM",P10="KON"),COUNTIFS($M$2:$M$1000,M10,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q10)+COUNTIFS($M$1:M9,M10,$P$1:P9,"RAM",$Q$1:Q9,Q10)+COUNTIFS($M$2:$M$1000,M10,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q10)+COUNTIFS($M$1:M9,M10,$P$1:P9,"KON",$Q$1:Q9,Q10)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M11" s="1" t="n">
+        <v>99008188</v>
+      </c>
       <c r="N11" s="1" t="n">
         <v>1487522</v>
       </c>
@@ -695,11 +719,14 @@
         <v>128</v>
       </c>
       <c r="T11" s="1" t="str">
-        <f aca="false">IF(AND(OR(P11="RAM",P11="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M10&lt;&gt;"")*($M$1:M10&lt;&gt;LOOKUP(2,1/($M$2:M11&lt;&gt;""),$M$2:M11))),ROW($M$1:M10)),1)+MATCH(LOOKUP(2,1/($M$2:M11&lt;&gt;""),$M$2:M11),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M10&lt;&gt;"")*($M$1:M10&lt;&gt;LOOKUP(2,1/($M$2:M11&lt;&gt;""),$M$2:M11))),ROW($M$1:M10)),1)+1):M11,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M12:$M$1001&lt;&gt;"")*(M12:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M11&lt;&gt;""),$M$2:M11)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q11)+($Q$2:$Q$1000=Q11)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P11="RAM",P11="KON"),COUNTIFS($M$2:$M$1000,M11,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q11)+COUNTIFS($M$1:M10,M11,$P$1:P10,"RAM",$Q$1:Q10,Q11)+COUNTIFS($M$2:$M$1000,M11,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q11)+COUNTIFS($M$1:M10,M11,$P$1:P10,"KON",$Q$1:Q10,Q11)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M12" s="1" t="n">
+        <v>99008188</v>
+      </c>
       <c r="N12" s="1" t="n">
         <v>145211</v>
       </c>
@@ -719,11 +746,14 @@
         <v>59</v>
       </c>
       <c r="T12" s="1" t="str">
-        <f aca="false">IF(AND(OR(P12="RAM",P12="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M11&lt;&gt;"")*($M$1:M11&lt;&gt;LOOKUP(2,1/($M$2:M12&lt;&gt;""),$M$2:M12))),ROW($M$1:M11)),1)+MATCH(LOOKUP(2,1/($M$2:M12&lt;&gt;""),$M$2:M12),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M11&lt;&gt;"")*($M$1:M11&lt;&gt;LOOKUP(2,1/($M$2:M12&lt;&gt;""),$M$2:M12))),ROW($M$1:M11)),1)+1):M12,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M13:$M$1001&lt;&gt;"")*(M13:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M12&lt;&gt;""),$M$2:M12)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q12)+($Q$2:$Q$1000=Q12)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P12="RAM",P12="KON"),COUNTIFS($M$2:$M$1000,M12,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q12)+COUNTIFS($M$1:M11,M12,$P$1:P11,"RAM",$Q$1:Q11,Q12)+COUNTIFS($M$2:$M$1000,M12,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q12)+COUNTIFS($M$1:M11,M12,$P$1:P11,"KON",$Q$1:Q11,Q12)=0),"Выбрать","")</f>
         <v>Выбрать</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M13" s="1" t="n">
+        <v>99008188</v>
+      </c>
       <c r="N13" s="1" t="n">
         <v>1177852</v>
       </c>
@@ -743,11 +773,14 @@
         <v>118</v>
       </c>
       <c r="T13" s="1" t="str">
-        <f aca="false">IF(AND(OR(P13="RAM",P13="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M12&lt;&gt;"")*($M$1:M12&lt;&gt;LOOKUP(2,1/($M$2:M13&lt;&gt;""),$M$2:M13))),ROW($M$1:M12)),1)+MATCH(LOOKUP(2,1/($M$2:M13&lt;&gt;""),$M$2:M13),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M12&lt;&gt;"")*($M$1:M12&lt;&gt;LOOKUP(2,1/($M$2:M13&lt;&gt;""),$M$2:M13))),ROW($M$1:M12)),1)+1):M13,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M14:$M$1001&lt;&gt;"")*(M14:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M13&lt;&gt;""),$M$2:M13)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q13)+($Q$2:$Q$1000=Q13)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P13="RAM",P13="KON"),COUNTIFS($M$2:$M$1000,M13,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q13)+COUNTIFS($M$1:M12,M13,$P$1:P12,"RAM",$Q$1:Q12,Q13)+COUNTIFS($M$2:$M$1000,M13,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q13)+COUNTIFS($M$1:M12,M13,$P$1:P12,"KON",$Q$1:Q12,Q13)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M14" s="1" t="n">
+        <v>99008188</v>
+      </c>
       <c r="N14" s="1" t="n">
         <v>445221</v>
       </c>
@@ -767,11 +800,14 @@
         <v>81</v>
       </c>
       <c r="T14" s="1" t="str">
-        <f aca="false">IF(AND(OR(P14="RAM",P14="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M13&lt;&gt;"")*($M$1:M13&lt;&gt;LOOKUP(2,1/($M$2:M14&lt;&gt;""),$M$2:M14))),ROW($M$1:M13)),1)+MATCH(LOOKUP(2,1/($M$2:M14&lt;&gt;""),$M$2:M14),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M13&lt;&gt;"")*($M$1:M13&lt;&gt;LOOKUP(2,1/($M$2:M14&lt;&gt;""),$M$2:M14))),ROW($M$1:M13)),1)+1):M14,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M15:$M$1001&lt;&gt;"")*(M15:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M14&lt;&gt;""),$M$2:M14)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q14)+($Q$2:$Q$1000=Q14)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P14="RAM",P14="KON"),COUNTIFS($M$2:$M$1000,M14,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q14)+COUNTIFS($M$1:M13,M14,$P$1:P13,"RAM",$Q$1:Q13,Q14)+COUNTIFS($M$2:$M$1000,M14,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q14)+COUNTIFS($M$1:M13,M14,$P$1:P13,"KON",$Q$1:Q13,Q14)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M15" s="1" t="n">
+        <v>99008188</v>
+      </c>
       <c r="N15" s="1" t="n">
         <v>441155</v>
       </c>
@@ -791,11 +827,14 @@
         <v>118</v>
       </c>
       <c r="T15" s="1" t="str">
-        <f aca="false">IF(AND(OR(P15="RAM",P15="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M14&lt;&gt;"")*($M$1:M14&lt;&gt;LOOKUP(2,1/($M$2:M15&lt;&gt;""),$M$2:M15))),ROW($M$1:M14)),1)+MATCH(LOOKUP(2,1/($M$2:M15&lt;&gt;""),$M$2:M15),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M14&lt;&gt;"")*($M$1:M14&lt;&gt;LOOKUP(2,1/($M$2:M15&lt;&gt;""),$M$2:M15))),ROW($M$1:M14)),1)+1):M15,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M16:$M$1001&lt;&gt;"")*(M16:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M15&lt;&gt;""),$M$2:M15)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q15)+($Q$2:$Q$1000=Q15)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P15="RAM",P15="KON"),COUNTIFS($M$2:$M$1000,M15,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q15)+COUNTIFS($M$1:M14,M15,$P$1:P14,"RAM",$Q$1:Q14,Q15)+COUNTIFS($M$2:$M$1000,M15,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q15)+COUNTIFS($M$1:M14,M15,$P$1:P14,"KON",$Q$1:Q14,Q15)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M16" s="1" t="n">
+        <v>99008188</v>
+      </c>
       <c r="N16" s="1" t="n">
         <v>155221</v>
       </c>
@@ -815,11 +854,14 @@
         <v>128</v>
       </c>
       <c r="T16" s="1" t="str">
-        <f aca="false">IF(AND(OR(P16="RAM",P16="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M15&lt;&gt;"")*($M$1:M15&lt;&gt;LOOKUP(2,1/($M$2:M16&lt;&gt;""),$M$2:M16))),ROW($M$1:M15)),1)+MATCH(LOOKUP(2,1/($M$2:M16&lt;&gt;""),$M$2:M16),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M15&lt;&gt;"")*($M$1:M15&lt;&gt;LOOKUP(2,1/($M$2:M16&lt;&gt;""),$M$2:M16))),ROW($M$1:M15)),1)+1):M16,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M17:$M$1001&lt;&gt;"")*(M17:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M16&lt;&gt;""),$M$2:M16)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q16)+($Q$2:$Q$1000=Q16)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P16="RAM",P16="KON"),COUNTIFS($M$2:$M$1000,M16,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q16)+COUNTIFS($M$1:M15,M16,$P$1:P15,"RAM",$Q$1:Q15,Q16)+COUNTIFS($M$2:$M$1000,M16,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q16)+COUNTIFS($M$1:M15,M16,$P$1:P15,"KON",$Q$1:Q15,Q16)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M17" s="1" t="n">
+        <v>99008188</v>
+      </c>
       <c r="N17" s="1" t="n">
         <v>5444445</v>
       </c>
@@ -841,7 +883,7 @@
         <v>#N/A</v>
       </c>
       <c r="T17" s="1" t="str">
-        <f aca="false">IF(AND(OR(P17="RAM",P17="KON"),SUMPRODUCT((ROW($P$2:$P$1000)&gt;=(IFERROR(LOOKUP(2,1/(($M$1:M16&lt;&gt;"")*($M$1:M16&lt;&gt;LOOKUP(2,1/($M$2:M17&lt;&gt;""),$M$2:M17))),ROW($M$1:M16)),1)+MATCH(LOOKUP(2,1/($M$2:M17&lt;&gt;""),$M$2:M17),INDEX($M:$M,IFERROR(LOOKUP(2,1/(($M$1:M16&lt;&gt;"")*($M$1:M16&lt;&gt;LOOKUP(2,1/($M$2:M17&lt;&gt;""),$M$2:M17))),ROW($M$1:M16)),1)+1):M17,0)))*(ROW($P$2:$P$1000)&lt;=IFERROR(MATCH(1,INDEX((M18:$M$1001&lt;&gt;"")*(M18:$M$1001&lt;&gt;LOOKUP(2,1/($M$2:M17&lt;&gt;""),$M$2:M17)),0),0)+ROW()-1,1000))*(($P$2:$P$1000="RAM")+($P$2:$P$1000="KON"))*(($Q$2:$Q$1000&lt;Q17)+($Q$2:$Q$1000=Q17)*(ROW($Q$2:$Q$1000)&lt;ROW())))=0),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P17="RAM",P17="KON"),COUNTIFS($M$2:$M$1000,M17,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q17)+COUNTIFS($M$1:M16,M17,$P$1:P16,"RAM",$Q$1:Q16,Q17)+COUNTIFS($M$2:$M$1000,M17,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q17)+COUNTIFS($M$1:M16,M17,$P$1:P16,"KON",$Q$1:Q16,Q17)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fall back to lowest price when an ID group has no contract
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFaw3CrmucU3qXrStYrfnC
</commit_message>
<xml_diff>
--- a/Выбор_по_договору_ID.xlsx
+++ b/Выбор_по_договору_ID.xlsx
@@ -474,7 +474,7 @@
         <v>158</v>
       </c>
       <c r="T2" s="1" t="str">
-        <f aca="false">IF(AND(OR(P2="RAM",P2="KON"),COUNTIFS($M$2:$M$1000,M2,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q2)+COUNTIFS($M$1:M1,M2,$P$1:P1,"RAM",$Q$1:Q1,Q2)+COUNTIFS($M$2:$M$1000,M2,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q2)+COUNTIFS($M$1:M1,M2,$P$1:P1,"KON",$Q$1:Q1,Q2)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M2,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M2,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P2="RAM",P2="KON"),COUNTIFS($M$2:$M$1000,M2,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q2)+COUNTIFS($M$1:M1,M2,$P$1:P1,"RAM",$Q$1:Q1,Q2)+COUNTIFS($M$2:$M$1000,M2,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q2)+COUNTIFS($M$1:M1,M2,$P$1:P1,"KON",$Q$1:Q1,Q2)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M2,$Q$2:$Q$1000,"&lt;"&amp;Q2)+COUNTIFS($M$1:M1,M2,$Q$1:Q1,Q2)=0,"Выбрать",""))</f>
         <v/>
       </c>
     </row>
@@ -501,7 +501,7 @@
         <v>128</v>
       </c>
       <c r="T3" s="1" t="str">
-        <f aca="false">IF(AND(OR(P3="RAM",P3="KON"),COUNTIFS($M$2:$M$1000,M3,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q3)+COUNTIFS($M$1:M2,M3,$P$1:P2,"RAM",$Q$1:Q2,Q3)+COUNTIFS($M$2:$M$1000,M3,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q3)+COUNTIFS($M$1:M2,M3,$P$1:P2,"KON",$Q$1:Q2,Q3)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M3,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M3,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P3="RAM",P3="KON"),COUNTIFS($M$2:$M$1000,M3,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q3)+COUNTIFS($M$1:M2,M3,$P$1:P2,"RAM",$Q$1:Q2,Q3)+COUNTIFS($M$2:$M$1000,M3,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q3)+COUNTIFS($M$1:M2,M3,$P$1:P2,"KON",$Q$1:Q2,Q3)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M3,$Q$2:$Q$1000,"&lt;"&amp;Q3)+COUNTIFS($M$1:M2,M3,$Q$1:Q2,Q3)=0,"Выбрать",""))</f>
         <v/>
       </c>
     </row>
@@ -528,7 +528,7 @@
         <v>59</v>
       </c>
       <c r="T4" s="1" t="str">
-        <f aca="false">IF(AND(OR(P4="RAM",P4="KON"),COUNTIFS($M$2:$M$1000,M4,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q4)+COUNTIFS($M$1:M3,M4,$P$1:P3,"RAM",$Q$1:Q3,Q4)+COUNTIFS($M$2:$M$1000,M4,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q4)+COUNTIFS($M$1:M3,M4,$P$1:P3,"KON",$Q$1:Q3,Q4)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M4,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M4,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P4="RAM",P4="KON"),COUNTIFS($M$2:$M$1000,M4,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q4)+COUNTIFS($M$1:M3,M4,$P$1:P3,"RAM",$Q$1:Q3,Q4)+COUNTIFS($M$2:$M$1000,M4,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q4)+COUNTIFS($M$1:M3,M4,$P$1:P3,"KON",$Q$1:Q3,Q4)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M4,$Q$2:$Q$1000,"&lt;"&amp;Q4)+COUNTIFS($M$1:M3,M4,$Q$1:Q3,Q4)=0,"Выбрать",""))</f>
         <v>Выбрать</v>
       </c>
     </row>
@@ -555,7 +555,7 @@
         <v>118</v>
       </c>
       <c r="T5" s="1" t="str">
-        <f aca="false">IF(AND(OR(P5="RAM",P5="KON"),COUNTIFS($M$2:$M$1000,M5,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q5)+COUNTIFS($M$1:M4,M5,$P$1:P4,"RAM",$Q$1:Q4,Q5)+COUNTIFS($M$2:$M$1000,M5,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q5)+COUNTIFS($M$1:M4,M5,$P$1:P4,"KON",$Q$1:Q4,Q5)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M5,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M5,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P5="RAM",P5="KON"),COUNTIFS($M$2:$M$1000,M5,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q5)+COUNTIFS($M$1:M4,M5,$P$1:P4,"RAM",$Q$1:Q4,Q5)+COUNTIFS($M$2:$M$1000,M5,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q5)+COUNTIFS($M$1:M4,M5,$P$1:P4,"KON",$Q$1:Q4,Q5)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M5,$Q$2:$Q$1000,"&lt;"&amp;Q5)+COUNTIFS($M$1:M4,M5,$Q$1:Q4,Q5)=0,"Выбрать",""))</f>
         <v/>
       </c>
     </row>
@@ -582,7 +582,7 @@
         <v>81</v>
       </c>
       <c r="T6" s="1" t="str">
-        <f aca="false">IF(AND(OR(P6="RAM",P6="KON"),COUNTIFS($M$2:$M$1000,M6,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q6)+COUNTIFS($M$1:M5,M6,$P$1:P5,"RAM",$Q$1:Q5,Q6)+COUNTIFS($M$2:$M$1000,M6,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q6)+COUNTIFS($M$1:M5,M6,$P$1:P5,"KON",$Q$1:Q5,Q6)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M6,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M6,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P6="RAM",P6="KON"),COUNTIFS($M$2:$M$1000,M6,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q6)+COUNTIFS($M$1:M5,M6,$P$1:P5,"RAM",$Q$1:Q5,Q6)+COUNTIFS($M$2:$M$1000,M6,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q6)+COUNTIFS($M$1:M5,M6,$P$1:P5,"KON",$Q$1:Q5,Q6)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M6,$Q$2:$Q$1000,"&lt;"&amp;Q6)+COUNTIFS($M$1:M5,M6,$Q$1:Q5,Q6)=0,"Выбрать",""))</f>
         <v/>
       </c>
     </row>
@@ -609,7 +609,7 @@
         <v>118</v>
       </c>
       <c r="T7" s="1" t="str">
-        <f aca="false">IF(AND(OR(P7="RAM",P7="KON"),COUNTIFS($M$2:$M$1000,M7,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q7)+COUNTIFS($M$1:M6,M7,$P$1:P6,"RAM",$Q$1:Q6,Q7)+COUNTIFS($M$2:$M$1000,M7,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q7)+COUNTIFS($M$1:M6,M7,$P$1:P6,"KON",$Q$1:Q6,Q7)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M7,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M7,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P7="RAM",P7="KON"),COUNTIFS($M$2:$M$1000,M7,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q7)+COUNTIFS($M$1:M6,M7,$P$1:P6,"RAM",$Q$1:Q6,Q7)+COUNTIFS($M$2:$M$1000,M7,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q7)+COUNTIFS($M$1:M6,M7,$P$1:P6,"KON",$Q$1:Q6,Q7)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M7,$Q$2:$Q$1000,"&lt;"&amp;Q7)+COUNTIFS($M$1:M6,M7,$Q$1:Q6,Q7)=0,"Выбрать",""))</f>
         <v/>
       </c>
     </row>
@@ -636,7 +636,7 @@
         <v>128</v>
       </c>
       <c r="T8" s="1" t="str">
-        <f aca="false">IF(AND(OR(P8="RAM",P8="KON"),COUNTIFS($M$2:$M$1000,M8,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q8)+COUNTIFS($M$1:M7,M8,$P$1:P7,"RAM",$Q$1:Q7,Q8)+COUNTIFS($M$2:$M$1000,M8,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q8)+COUNTIFS($M$1:M7,M8,$P$1:P7,"KON",$Q$1:Q7,Q8)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M8,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M8,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P8="RAM",P8="KON"),COUNTIFS($M$2:$M$1000,M8,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q8)+COUNTIFS($M$1:M7,M8,$P$1:P7,"RAM",$Q$1:Q7,Q8)+COUNTIFS($M$2:$M$1000,M8,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q8)+COUNTIFS($M$1:M7,M8,$P$1:P7,"KON",$Q$1:Q7,Q8)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M8,$Q$2:$Q$1000,"&lt;"&amp;Q8)+COUNTIFS($M$1:M7,M8,$Q$1:Q7,Q8)=0,"Выбрать",""))</f>
         <v/>
       </c>
     </row>
@@ -665,7 +665,7 @@
         <v>#N/A</v>
       </c>
       <c r="T9" s="1" t="str">
-        <f aca="false">IF(AND(OR(P9="RAM",P9="KON"),COUNTIFS($M$2:$M$1000,M9,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q9)+COUNTIFS($M$1:M8,M9,$P$1:P8,"RAM",$Q$1:Q8,Q9)+COUNTIFS($M$2:$M$1000,M9,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q9)+COUNTIFS($M$1:M8,M9,$P$1:P8,"KON",$Q$1:Q8,Q9)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M9,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M9,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P9="RAM",P9="KON"),COUNTIFS($M$2:$M$1000,M9,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q9)+COUNTIFS($M$1:M8,M9,$P$1:P8,"RAM",$Q$1:Q8,Q9)+COUNTIFS($M$2:$M$1000,M9,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q9)+COUNTIFS($M$1:M8,M9,$P$1:P8,"KON",$Q$1:Q8,Q9)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M9,$Q$2:$Q$1000,"&lt;"&amp;Q9)+COUNTIFS($M$1:M8,M9,$Q$1:Q8,Q9)=0,"Выбрать",""))</f>
         <v/>
       </c>
     </row>
@@ -692,7 +692,7 @@
         <v>158</v>
       </c>
       <c r="T10" s="1" t="str">
-        <f aca="false">IF(AND(OR(P10="RAM",P10="KON"),COUNTIFS($M$2:$M$1000,M10,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q10)+COUNTIFS($M$1:M9,M10,$P$1:P9,"RAM",$Q$1:Q9,Q10)+COUNTIFS($M$2:$M$1000,M10,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q10)+COUNTIFS($M$1:M9,M10,$P$1:P9,"KON",$Q$1:Q9,Q10)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M10,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M10,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P10="RAM",P10="KON"),COUNTIFS($M$2:$M$1000,M10,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q10)+COUNTIFS($M$1:M9,M10,$P$1:P9,"RAM",$Q$1:Q9,Q10)+COUNTIFS($M$2:$M$1000,M10,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q10)+COUNTIFS($M$1:M9,M10,$P$1:P9,"KON",$Q$1:Q9,Q10)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M10,$Q$2:$Q$1000,"&lt;"&amp;Q10)+COUNTIFS($M$1:M9,M10,$Q$1:Q9,Q10)=0,"Выбрать",""))</f>
         <v/>
       </c>
     </row>
@@ -719,7 +719,7 @@
         <v>128</v>
       </c>
       <c r="T11" s="1" t="str">
-        <f aca="false">IF(AND(OR(P11="RAM",P11="KON"),COUNTIFS($M$2:$M$1000,M11,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q11)+COUNTIFS($M$1:M10,M11,$P$1:P10,"RAM",$Q$1:Q10,Q11)+COUNTIFS($M$2:$M$1000,M11,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q11)+COUNTIFS($M$1:M10,M11,$P$1:P10,"KON",$Q$1:Q10,Q11)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M11,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M11,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P11="RAM",P11="KON"),COUNTIFS($M$2:$M$1000,M11,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q11)+COUNTIFS($M$1:M10,M11,$P$1:P10,"RAM",$Q$1:Q10,Q11)+COUNTIFS($M$2:$M$1000,M11,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q11)+COUNTIFS($M$1:M10,M11,$P$1:P10,"KON",$Q$1:Q10,Q11)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M11,$Q$2:$Q$1000,"&lt;"&amp;Q11)+COUNTIFS($M$1:M10,M11,$Q$1:Q10,Q11)=0,"Выбрать",""))</f>
         <v/>
       </c>
     </row>
@@ -746,7 +746,7 @@
         <v>59</v>
       </c>
       <c r="T12" s="1" t="str">
-        <f aca="false">IF(AND(OR(P12="RAM",P12="KON"),COUNTIFS($M$2:$M$1000,M12,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q12)+COUNTIFS($M$1:M11,M12,$P$1:P11,"RAM",$Q$1:Q11,Q12)+COUNTIFS($M$2:$M$1000,M12,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q12)+COUNTIFS($M$1:M11,M12,$P$1:P11,"KON",$Q$1:Q11,Q12)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M12,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M12,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P12="RAM",P12="KON"),COUNTIFS($M$2:$M$1000,M12,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q12)+COUNTIFS($M$1:M11,M12,$P$1:P11,"RAM",$Q$1:Q11,Q12)+COUNTIFS($M$2:$M$1000,M12,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q12)+COUNTIFS($M$1:M11,M12,$P$1:P11,"KON",$Q$1:Q11,Q12)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M12,$Q$2:$Q$1000,"&lt;"&amp;Q12)+COUNTIFS($M$1:M11,M12,$Q$1:Q11,Q12)=0,"Выбрать",""))</f>
         <v>Выбрать</v>
       </c>
     </row>
@@ -773,7 +773,7 @@
         <v>118</v>
       </c>
       <c r="T13" s="1" t="str">
-        <f aca="false">IF(AND(OR(P13="RAM",P13="KON"),COUNTIFS($M$2:$M$1000,M13,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q13)+COUNTIFS($M$1:M12,M13,$P$1:P12,"RAM",$Q$1:Q12,Q13)+COUNTIFS($M$2:$M$1000,M13,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q13)+COUNTIFS($M$1:M12,M13,$P$1:P12,"KON",$Q$1:Q12,Q13)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M13,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M13,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P13="RAM",P13="KON"),COUNTIFS($M$2:$M$1000,M13,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q13)+COUNTIFS($M$1:M12,M13,$P$1:P12,"RAM",$Q$1:Q12,Q13)+COUNTIFS($M$2:$M$1000,M13,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q13)+COUNTIFS($M$1:M12,M13,$P$1:P12,"KON",$Q$1:Q12,Q13)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M13,$Q$2:$Q$1000,"&lt;"&amp;Q13)+COUNTIFS($M$1:M12,M13,$Q$1:Q12,Q13)=0,"Выбрать",""))</f>
         <v/>
       </c>
     </row>
@@ -800,7 +800,7 @@
         <v>81</v>
       </c>
       <c r="T14" s="1" t="str">
-        <f aca="false">IF(AND(OR(P14="RAM",P14="KON"),COUNTIFS($M$2:$M$1000,M14,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q14)+COUNTIFS($M$1:M13,M14,$P$1:P13,"RAM",$Q$1:Q13,Q14)+COUNTIFS($M$2:$M$1000,M14,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q14)+COUNTIFS($M$1:M13,M14,$P$1:P13,"KON",$Q$1:Q13,Q14)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M14,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M14,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P14="RAM",P14="KON"),COUNTIFS($M$2:$M$1000,M14,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q14)+COUNTIFS($M$1:M13,M14,$P$1:P13,"RAM",$Q$1:Q13,Q14)+COUNTIFS($M$2:$M$1000,M14,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q14)+COUNTIFS($M$1:M13,M14,$P$1:P13,"KON",$Q$1:Q13,Q14)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M14,$Q$2:$Q$1000,"&lt;"&amp;Q14)+COUNTIFS($M$1:M13,M14,$Q$1:Q13,Q14)=0,"Выбрать",""))</f>
         <v/>
       </c>
     </row>
@@ -827,7 +827,7 @@
         <v>118</v>
       </c>
       <c r="T15" s="1" t="str">
-        <f aca="false">IF(AND(OR(P15="RAM",P15="KON"),COUNTIFS($M$2:$M$1000,M15,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q15)+COUNTIFS($M$1:M14,M15,$P$1:P14,"RAM",$Q$1:Q14,Q15)+COUNTIFS($M$2:$M$1000,M15,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q15)+COUNTIFS($M$1:M14,M15,$P$1:P14,"KON",$Q$1:Q14,Q15)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M15,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M15,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P15="RAM",P15="KON"),COUNTIFS($M$2:$M$1000,M15,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q15)+COUNTIFS($M$1:M14,M15,$P$1:P14,"RAM",$Q$1:Q14,Q15)+COUNTIFS($M$2:$M$1000,M15,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q15)+COUNTIFS($M$1:M14,M15,$P$1:P14,"KON",$Q$1:Q14,Q15)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M15,$Q$2:$Q$1000,"&lt;"&amp;Q15)+COUNTIFS($M$1:M14,M15,$Q$1:Q14,Q15)=0,"Выбрать",""))</f>
         <v/>
       </c>
     </row>
@@ -854,7 +854,7 @@
         <v>128</v>
       </c>
       <c r="T16" s="1" t="str">
-        <f aca="false">IF(AND(OR(P16="RAM",P16="KON"),COUNTIFS($M$2:$M$1000,M16,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q16)+COUNTIFS($M$1:M15,M16,$P$1:P15,"RAM",$Q$1:Q15,Q16)+COUNTIFS($M$2:$M$1000,M16,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q16)+COUNTIFS($M$1:M15,M16,$P$1:P15,"KON",$Q$1:Q15,Q16)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M16,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M16,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P16="RAM",P16="KON"),COUNTIFS($M$2:$M$1000,M16,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q16)+COUNTIFS($M$1:M15,M16,$P$1:P15,"RAM",$Q$1:Q15,Q16)+COUNTIFS($M$2:$M$1000,M16,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q16)+COUNTIFS($M$1:M15,M16,$P$1:P15,"KON",$Q$1:Q15,Q16)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M16,$Q$2:$Q$1000,"&lt;"&amp;Q16)+COUNTIFS($M$1:M15,M16,$Q$1:Q15,Q16)=0,"Выбрать",""))</f>
         <v/>
       </c>
     </row>
@@ -883,7 +883,7 @@
         <v>#N/A</v>
       </c>
       <c r="T17" s="1" t="str">
-        <f aca="false">IF(AND(OR(P17="RAM",P17="KON"),COUNTIFS($M$2:$M$1000,M17,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q17)+COUNTIFS($M$1:M16,M17,$P$1:P16,"RAM",$Q$1:Q16,Q17)+COUNTIFS($M$2:$M$1000,M17,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q17)+COUNTIFS($M$1:M16,M17,$P$1:P16,"KON",$Q$1:Q16,Q17)=0),"Выбрать","")</f>
+        <f aca="false">IF(COUNTIFS($M$2:$M$1000,M17,$P$2:$P$1000,"RAM")+COUNTIFS($M$2:$M$1000,M17,$P$2:$P$1000,"KON")&gt;0,IF(AND(OR(P17="RAM",P17="KON"),COUNTIFS($M$2:$M$1000,M17,$P$2:$P$1000,"RAM",$Q$2:$Q$1000,"&lt;"&amp;Q17)+COUNTIFS($M$1:M16,M17,$P$1:P16,"RAM",$Q$1:Q16,Q17)+COUNTIFS($M$2:$M$1000,M17,$P$2:$P$1000,"KON",$Q$2:$Q$1000,"&lt;"&amp;Q17)+COUNTIFS($M$1:M16,M17,$P$1:P16,"KON",$Q$1:Q16,Q17)=0),"Выбрать",""),IF(COUNTIFS($M$2:$M$1000,M17,$Q$2:$Q$1000,"&lt;"&amp;Q17)+COUNTIFS($M$1:M16,M17,$Q$1:Q16,Q17)=0,"Выбрать",""))</f>
         <v/>
       </c>
     </row>

</xml_diff>